<commit_message>
Follow-up: user's renamed columns + Principal Contact (Details on each card, as on the tour page); one value per line (lists refused loudly instead of silently using one value); 5th week of month; version followup-2026-10-08.4
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GfyZEqTUWy44eCLhgpngu7
</commit_message>
<xml_diff>
--- a/docs/followup/sample-followup-sheet.xlsx
+++ b/docs/followup/sample-followup-sheet.xlsx
@@ -164,7 +164,7 @@
     </comment>
     <comment ref="B1" authorId="0" shapeId="0">
       <text>
-        <t>Monday...Sunday, or Every day (Daily lines).</t>
+        <t>One day: Monday...Sunday, or Every day (Daily lines). Several days = one line each.</t>
       </text>
     </comment>
     <comment ref="C1" authorId="0" shapeId="0">
@@ -184,12 +184,12 @@
     </comment>
     <comment ref="F1" authorId="0" shapeId="0">
       <text>
-        <t>Monthly, same weekday only: 1st, 2nd, 3rd, 4th or last.</t>
+        <t>Monthly, same weekday only: one of 1st, 2nd, 3rd, 4th, 5th (months without one are skipped) or last.</t>
       </text>
     </comment>
     <comment ref="G1" authorId="0" shapeId="0">
       <text>
-        <t>Monthly, same date only: 1 to 31. Months without that date are skipped.</t>
+        <t>Monthly, same date only: one number, 1 to 31. Months without that date are skipped.</t>
       </text>
     </comment>
     <comment ref="J1" authorId="0" shapeId="0">
@@ -213,6 +213,11 @@
       </text>
     </comment>
     <comment ref="N1" authorId="0" shapeId="0">
+      <text>
+        <t>Principal name + phone, shown on each date under Details.</t>
+      </text>
+    </comment>
+    <comment ref="O1" authorId="0" shapeId="0">
       <text>
         <t>Organiser name + phone, shown when release is closed.</t>
       </text>
@@ -244,25 +249,30 @@
     </comment>
     <comment ref="K1" authorId="0" shapeId="0">
       <text>
-        <t>Open or Cancelled. To drop a date, set Cancelled (do not delete the row).</t>
+        <t>Organisers may change.</t>
       </text>
     </comment>
     <comment ref="L1" authorId="0" shapeId="0">
       <text>
-        <t>Written by the page. Fix by hand only when needed.</t>
+        <t>Open or Cancelled. To drop a date, set Cancelled (do not delete the row).</t>
       </text>
     </comment>
     <comment ref="M1" authorId="0" shapeId="0">
       <text>
-        <t>Written by the page.</t>
+        <t>Written by the page. Fix by hand only when needed.</t>
       </text>
     </comment>
     <comment ref="N1" authorId="0" shapeId="0">
       <text>
+        <t>Written by the page.</t>
+      </text>
+    </comment>
+    <comment ref="O1" authorId="0" shapeId="0">
+      <text>
         <t>Written by the WhatsApp-list tool.</t>
       </text>
     </comment>
-    <comment ref="O1" authorId="0" shapeId="0">
+    <comment ref="P1" authorId="0" shapeId="0">
       <text>
         <t>Organisers may change.</t>
       </text>
@@ -560,7 +570,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A15"/>
+  <dimension ref="A1:A16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="140" customWidth="1" min="1" max="1"/>
@@ -586,78 +596,85 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">   Leave "Line ID" empty for new lines: the script fills it in. Type times with AM/PM. Pick Day, Frequency and Week of month from the lists.</t>
+          <t xml:space="preserve">   Leave "Line ID" empty for new lines: the script fills it in. Type times with AM/PM. Pick Day of the Week, Frequency and Week of month from the lists.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>Slots: made by the script from Program plan (Program -&gt; Update slots now), one row per date. Do not type dates here.</t>
+          <t xml:space="preserve">   One value per line: for Monday and Thursday, or the 1st and 3rd Saturday, type two lines (a list is refused and listed in Update report).</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">   Organisers may change Status (Open/Cancelled), Places, Contact and Notes. Volunteers and Still needed are written by the page.</t>
+          <t>Slots: made by the script from Program plan (Program -&gt; Update slots now), one row per date. Do not type dates here.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">   Here: Asha Rao booked herself and Ravi Kumar (via Asha Rao) for 4 Saturdays; 24 Oct is Cancelled to show the notice.</t>
+          <t xml:space="preserve">   Organisers may change Status (Open/Cancelled), Volunteers Needed, Principal Contact, Sahaji Contact and Notes. Volunteers and Still needed are written by the page.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>Speakers: the names volunteers can pick from (Sr. No., Speaker, Mobile). Meena Iyer has no mobile yet, to show the first-time mobile box.</t>
+          <t xml:space="preserve">   Here: Asha Rao booked herself and Ravi Kumar (via Asha Rao) for 4 Saturdays; 24 Oct is Cancelled to show the notice.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
+          <t>Speakers: the names volunteers can pick from (Sr. No., Speaker, Mobile). Meena Iyer has no mobile yet, to show the first-time mobile box.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
           <t>Update report: what the last "Update slots now" did and anything that needs you.</t>
         </is>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" s="2" t="inlineStr"/>
-    </row>
     <row r="11">
-      <c r="A11" s="2" t="inlineStr">
-        <is>
-          <t>To make a sample copy with real data: replace the rows under the titles in Program plan and Speakers with real ones</t>
-        </is>
-      </c>
+      <c r="A11" s="2" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">   (and clear the Line ID column). Slots, Volunteers and Update report can be left as they are, or emptied.</t>
+          <t>To make a sample copy with real data: replace the rows under the titles in Program plan and Speakers with real ones</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>Privacy: real mobile numbers are fine in your own copy. When you share a copy with Claude, it is kept out of the code repository;</t>
+          <t xml:space="preserve">   (and clear the Line ID column). Slots, Volunteers and Update report can be left as they are, or emptied.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">   you can also replace the last digits of the numbers if you prefer.</t>
+          <t>Privacy: real mobile numbers are fine in your own copy. When you share a copy with Claude, it is kept out of the code repository;</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   you can also replace the last digits of the numbers if you prefer.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
         <is>
           <t>Hover over a column title to read who fills it. Hover notes, drop-down lists, date and time formats match the live sheet.</t>
         </is>
@@ -674,11 +691,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O8"/>
+  <dimension ref="A1:P8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
-    <col width="11" customWidth="1" min="2" max="2"/>
+    <col width="15" customWidth="1" min="2" max="2"/>
     <col width="10" customWidth="1" min="3" max="3"/>
     <col width="10" customWidth="1" min="4" max="4"/>
     <col width="30" customWidth="1" min="5" max="5"/>
@@ -687,11 +704,12 @@
     <col width="20" customWidth="1" min="8" max="8"/>
     <col width="22" customWidth="1" min="9" max="9"/>
     <col width="28" customWidth="1" min="10" max="10"/>
-    <col width="8" customWidth="1" min="11" max="11"/>
+    <col width="10" customWidth="1" min="11" max="11"/>
     <col width="13" customWidth="1" min="12" max="12"/>
     <col width="13" customWidth="1" min="13" max="13"/>
-    <col width="20" customWidth="1" min="14" max="14"/>
-    <col width="34" customWidth="1" min="15" max="15"/>
+    <col width="24" customWidth="1" min="14" max="14"/>
+    <col width="20" customWidth="1" min="15" max="15"/>
+    <col width="34" customWidth="1" min="16" max="16"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -702,17 +720,17 @@
       </c>
       <c r="B1" s="3" t="inlineStr">
         <is>
-          <t>Day</t>
+          <t>Day of the Week</t>
         </is>
       </c>
       <c r="C1" s="3" t="inlineStr">
         <is>
-          <t>Start</t>
+          <t>Start Time</t>
         </is>
       </c>
       <c r="D1" s="3" t="inlineStr">
         <is>
-          <t>End</t>
+          <t>End Time</t>
         </is>
       </c>
       <c r="E1" s="3" t="inlineStr">
@@ -732,7 +750,7 @@
       </c>
       <c r="H1" s="3" t="inlineStr">
         <is>
-          <t>Centre</t>
+          <t>Institution Name</t>
         </is>
       </c>
       <c r="I1" s="3" t="inlineStr">
@@ -747,7 +765,7 @@
       </c>
       <c r="K1" s="3" t="inlineStr">
         <is>
-          <t>Places</t>
+          <t>Volunteers Needed</t>
         </is>
       </c>
       <c r="L1" s="3" t="inlineStr">
@@ -762,10 +780,15 @@
       </c>
       <c r="N1" s="3" t="inlineStr">
         <is>
-          <t>Contact</t>
+          <t>Principal Contact</t>
         </is>
       </c>
       <c r="O1" s="3" t="inlineStr">
+        <is>
+          <t>Sahaji Contact</t>
+        </is>
+      </c>
+      <c r="P1" s="3" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
@@ -819,6 +842,11 @@
       </c>
       <c r="N2" t="inlineStr">
         <is>
+          <t>Principal A 9000000011</t>
+        </is>
+      </c>
+      <c r="O2" t="inlineStr">
+        <is>
           <t>Lakshmi 9000000009</t>
         </is>
       </c>
@@ -871,6 +899,11 @@
       </c>
       <c r="N3" t="inlineStr">
         <is>
+          <t>Principal B 9000000012</t>
+        </is>
+      </c>
+      <c r="O3" t="inlineStr">
+        <is>
           <t>Lakshmi 9000000009</t>
         </is>
       </c>
@@ -918,6 +951,11 @@
       </c>
       <c r="N4" t="inlineStr">
         <is>
+          <t>Principal C 9000000013</t>
+        </is>
+      </c>
+      <c r="O4" t="inlineStr">
+        <is>
           <t>Suresh 9000000008</t>
         </is>
       </c>
@@ -967,10 +1005,15 @@
       </c>
       <c r="N5" t="inlineStr">
         <is>
+          <t>Principal D 9000000014</t>
+        </is>
+      </c>
+      <c r="O5" t="inlineStr">
+        <is>
           <t>Suresh 9000000008</t>
         </is>
       </c>
-      <c r="O5" t="inlineStr">
+      <c r="P5" t="inlineStr">
         <is>
           <t>No Until date: keeps 12 weeks ahead</t>
         </is>
@@ -1024,6 +1067,11 @@
       </c>
       <c r="N6" t="inlineStr">
         <is>
+          <t>Principal E 9000000015</t>
+        </is>
+      </c>
+      <c r="O6" t="inlineStr">
+        <is>
           <t>Lakshmi 9000000009</t>
         </is>
       </c>
@@ -1071,6 +1119,11 @@
       </c>
       <c r="N7" t="inlineStr">
         <is>
+          <t>Principal F 9000000016</t>
+        </is>
+      </c>
+      <c r="O7" t="inlineStr">
+        <is>
           <t>Suresh 9000000008</t>
         </is>
       </c>
@@ -1110,10 +1163,15 @@
       </c>
       <c r="N8" t="inlineStr">
         <is>
+          <t>Principal G 9000000017</t>
+        </is>
+      </c>
+      <c r="O8" t="inlineStr">
+        <is>
           <t>Lakshmi 9000000009</t>
         </is>
       </c>
-      <c r="O8" t="inlineStr">
+      <c r="P8" t="inlineStr">
         <is>
           <t>Children's Day programme</t>
         </is>
@@ -1128,7 +1186,7 @@
       <formula1>=Lists!$B$1:$B$7</formula1>
     </dataValidation>
     <dataValidation sqref="F2:F1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>=Lists!$C$1:$C$5</formula1>
+      <formula1>=Lists!$C$1:$C$6</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1142,7 +1200,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O82"/>
+  <dimension ref="A1:P82"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1153,13 +1211,14 @@
     <col width="20" customWidth="1" min="6" max="6"/>
     <col width="22" customWidth="1" min="7" max="7"/>
     <col width="28" customWidth="1" min="8" max="8"/>
-    <col width="20" customWidth="1" min="9" max="9"/>
-    <col width="8" customWidth="1" min="10" max="10"/>
-    <col width="11" customWidth="1" min="11" max="11"/>
-    <col width="36" customWidth="1" min="12" max="12"/>
-    <col width="8" customWidth="1" min="13" max="13"/>
-    <col width="14" customWidth="1" min="14" max="14"/>
-    <col width="16" customWidth="1" min="15" max="15"/>
+    <col width="24" customWidth="1" min="9" max="9"/>
+    <col width="20" customWidth="1" min="10" max="10"/>
+    <col width="10" customWidth="1" min="11" max="11"/>
+    <col width="11" customWidth="1" min="12" max="12"/>
+    <col width="36" customWidth="1" min="13" max="13"/>
+    <col width="8" customWidth="1" min="14" max="14"/>
+    <col width="14" customWidth="1" min="15" max="15"/>
+    <col width="16" customWidth="1" min="16" max="16"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1180,17 +1239,17 @@
       </c>
       <c r="D1" s="3" t="inlineStr">
         <is>
-          <t>Start</t>
+          <t>Start Time</t>
         </is>
       </c>
       <c r="E1" s="3" t="inlineStr">
         <is>
-          <t>End</t>
+          <t>End Time</t>
         </is>
       </c>
       <c r="F1" s="3" t="inlineStr">
         <is>
-          <t>Centre</t>
+          <t>Institution Name</t>
         </is>
       </c>
       <c r="G1" s="3" t="inlineStr">
@@ -1205,35 +1264,40 @@
       </c>
       <c r="I1" s="3" t="inlineStr">
         <is>
-          <t>Contact</t>
+          <t>Principal Contact</t>
         </is>
       </c>
       <c r="J1" s="3" t="inlineStr">
         <is>
-          <t>Places</t>
+          <t>Sahaji Contact</t>
         </is>
       </c>
       <c r="K1" s="3" t="inlineStr">
         <is>
+          <t>Volunteers Needed</t>
+        </is>
+      </c>
+      <c r="L1" s="3" t="inlineStr">
+        <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="L1" s="3" t="inlineStr">
+      <c r="M1" s="3" t="inlineStr">
         <is>
           <t>Volunteers</t>
         </is>
       </c>
-      <c r="M1" s="3" t="inlineStr">
+      <c r="N1" s="3" t="inlineStr">
         <is>
           <t>Still needed</t>
         </is>
       </c>
-      <c r="N1" s="3" t="inlineStr">
+      <c r="O1" s="3" t="inlineStr">
         <is>
           <t>Cancellation notice sent</t>
         </is>
       </c>
-      <c r="O1" s="3" t="inlineStr">
+      <c r="P1" s="3" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
@@ -1271,18 +1335,23 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
+          <t>Principal E 9000000015</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
           <t>Lakshmi 9000000009</t>
         </is>
       </c>
-      <c r="J2" t="n">
+      <c r="K2" t="n">
         <v>5</v>
       </c>
-      <c r="K2" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="M2" t="n">
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="N2" t="n">
         <v>5</v>
       </c>
     </row>
@@ -1323,24 +1392,29 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
+          <t>Principal A 9000000011</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
           <t>Lakshmi 9000000009</t>
         </is>
       </c>
-      <c r="J3" t="n">
+      <c r="K3" t="n">
         <v>4</v>
       </c>
-      <c r="K3" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="L3" s="7" t="inlineStr">
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="M3" s="7" t="inlineStr">
         <is>
           <t>Asha Rao 9000000001
 Ravi Kumar 9000000002 (via Asha Rao)</t>
         </is>
       </c>
-      <c r="M3" t="n">
+      <c r="N3" t="n">
         <v>2</v>
       </c>
     </row>
@@ -1381,18 +1455,23 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
+          <t>Principal B 9000000012</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
           <t>Lakshmi 9000000009</t>
         </is>
       </c>
-      <c r="J4" t="n">
-        <v>2</v>
-      </c>
-      <c r="K4" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="M4" t="n">
+      <c r="K4" t="n">
+        <v>2</v>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="N4" t="n">
         <v>2</v>
       </c>
     </row>
@@ -1433,23 +1512,28 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
+          <t>Principal C 9000000013</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
           <t>Suresh 9000000008</t>
         </is>
       </c>
-      <c r="J5" t="n">
-        <v>2</v>
-      </c>
-      <c r="K5" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
+      <c r="K5" t="n">
+        <v>2</v>
       </c>
       <c r="L5" t="inlineStr">
         <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
           <t>Gita Sharma 9000000004</t>
         </is>
       </c>
-      <c r="M5" t="n">
+      <c r="N5" t="n">
         <v>1</v>
       </c>
     </row>
@@ -1490,18 +1574,23 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
+          <t>Principal B 9000000012</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
           <t>Lakshmi 9000000009</t>
         </is>
       </c>
-      <c r="J6" t="n">
-        <v>2</v>
-      </c>
-      <c r="K6" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="M6" t="n">
+      <c r="K6" t="n">
+        <v>2</v>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="N6" t="n">
         <v>2</v>
       </c>
     </row>
@@ -1542,18 +1631,23 @@
       </c>
       <c r="I7" t="inlineStr">
         <is>
+          <t>Principal C 9000000013</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
           <t>Suresh 9000000008</t>
         </is>
       </c>
-      <c r="J7" t="n">
-        <v>2</v>
-      </c>
-      <c r="K7" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="M7" t="n">
+      <c r="K7" t="n">
+        <v>2</v>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="N7" t="n">
         <v>2</v>
       </c>
     </row>
@@ -1594,18 +1688,23 @@
       </c>
       <c r="I8" t="inlineStr">
         <is>
+          <t>Principal B 9000000012</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
           <t>Lakshmi 9000000009</t>
         </is>
       </c>
-      <c r="J8" t="n">
-        <v>2</v>
-      </c>
-      <c r="K8" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="M8" t="n">
+      <c r="K8" t="n">
+        <v>2</v>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="N8" t="n">
         <v>2</v>
       </c>
     </row>
@@ -1646,18 +1745,23 @@
       </c>
       <c r="I9" t="inlineStr">
         <is>
+          <t>Principal C 9000000013</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
           <t>Suresh 9000000008</t>
         </is>
       </c>
-      <c r="J9" t="n">
-        <v>2</v>
-      </c>
-      <c r="K9" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="M9" t="n">
+      <c r="K9" t="n">
+        <v>2</v>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="N9" t="n">
         <v>2</v>
       </c>
     </row>
@@ -1698,18 +1802,23 @@
       </c>
       <c r="I10" t="inlineStr">
         <is>
+          <t>Principal B 9000000012</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
           <t>Lakshmi 9000000009</t>
         </is>
       </c>
-      <c r="J10" t="n">
-        <v>2</v>
-      </c>
-      <c r="K10" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="M10" t="n">
+      <c r="K10" t="n">
+        <v>2</v>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="N10" t="n">
         <v>2</v>
       </c>
     </row>
@@ -1745,18 +1854,23 @@
       </c>
       <c r="I11" t="inlineStr">
         <is>
+          <t>Principal F 9000000016</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
           <t>Suresh 9000000008</t>
         </is>
       </c>
-      <c r="J11" t="n">
-        <v>2</v>
-      </c>
-      <c r="K11" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="M11" t="n">
+      <c r="K11" t="n">
+        <v>2</v>
+      </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="N11" t="n">
         <v>2</v>
       </c>
     </row>
@@ -1797,18 +1911,23 @@
       </c>
       <c r="I12" t="inlineStr">
         <is>
+          <t>Principal C 9000000013</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
           <t>Suresh 9000000008</t>
         </is>
       </c>
-      <c r="J12" t="n">
-        <v>2</v>
-      </c>
-      <c r="K12" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="M12" t="n">
+      <c r="K12" t="n">
+        <v>2</v>
+      </c>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="N12" t="n">
         <v>2</v>
       </c>
     </row>
@@ -1849,18 +1968,23 @@
       </c>
       <c r="I13" t="inlineStr">
         <is>
+          <t>Principal B 9000000012</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
           <t>Lakshmi 9000000009</t>
         </is>
       </c>
-      <c r="J13" t="n">
-        <v>2</v>
-      </c>
-      <c r="K13" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="M13" t="n">
+      <c r="K13" t="n">
+        <v>2</v>
+      </c>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="N13" t="n">
         <v>2</v>
       </c>
     </row>
@@ -1901,18 +2025,23 @@
       </c>
       <c r="I14" t="inlineStr">
         <is>
+          <t>Principal C 9000000013</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
           <t>Suresh 9000000008</t>
         </is>
       </c>
-      <c r="J14" t="n">
-        <v>2</v>
-      </c>
-      <c r="K14" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="M14" t="n">
+      <c r="K14" t="n">
+        <v>2</v>
+      </c>
+      <c r="L14" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="N14" t="n">
         <v>2</v>
       </c>
     </row>
@@ -1953,18 +2082,23 @@
       </c>
       <c r="I15" t="inlineStr">
         <is>
+          <t>Principal B 9000000012</t>
+        </is>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
           <t>Lakshmi 9000000009</t>
         </is>
       </c>
-      <c r="J15" t="n">
-        <v>2</v>
-      </c>
-      <c r="K15" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="M15" t="n">
+      <c r="K15" t="n">
+        <v>2</v>
+      </c>
+      <c r="L15" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="N15" t="n">
         <v>2</v>
       </c>
     </row>
@@ -2005,25 +2139,30 @@
       </c>
       <c r="I16" t="inlineStr">
         <is>
+          <t>Principal A 9000000011</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
           <t>Lakshmi 9000000009</t>
         </is>
       </c>
-      <c r="J16" t="n">
+      <c r="K16" t="n">
         <v>4</v>
       </c>
-      <c r="K16" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="L16" s="7" t="inlineStr">
+      <c r="L16" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="M16" s="7" t="inlineStr">
         <is>
           <t>Asha Rao 9000000001
 Ravi Kumar 9000000002 (via Asha Rao)
 Hari Prasad 9000000005</t>
         </is>
       </c>
-      <c r="M16" t="n">
+      <c r="N16" t="n">
         <v>1</v>
       </c>
     </row>
@@ -2064,18 +2203,23 @@
       </c>
       <c r="I17" t="inlineStr">
         <is>
+          <t>Principal B 9000000012</t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
           <t>Lakshmi 9000000009</t>
         </is>
       </c>
-      <c r="J17" t="n">
-        <v>2</v>
-      </c>
-      <c r="K17" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="M17" t="n">
+      <c r="K17" t="n">
+        <v>2</v>
+      </c>
+      <c r="L17" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="N17" t="n">
         <v>2</v>
       </c>
     </row>
@@ -2116,18 +2260,23 @@
       </c>
       <c r="I18" t="inlineStr">
         <is>
+          <t>Principal D 9000000014</t>
+        </is>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
           <t>Suresh 9000000008</t>
         </is>
       </c>
-      <c r="J18" t="n">
+      <c r="K18" t="n">
         <v>3</v>
       </c>
-      <c r="K18" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="M18" t="n">
+      <c r="L18" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="N18" t="n">
         <v>3</v>
       </c>
     </row>
@@ -2168,18 +2317,23 @@
       </c>
       <c r="I19" t="inlineStr">
         <is>
+          <t>Principal B 9000000012</t>
+        </is>
+      </c>
+      <c r="J19" t="inlineStr">
+        <is>
           <t>Lakshmi 9000000009</t>
         </is>
       </c>
-      <c r="J19" t="n">
-        <v>2</v>
-      </c>
-      <c r="K19" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="M19" t="n">
+      <c r="K19" t="n">
+        <v>2</v>
+      </c>
+      <c r="L19" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="N19" t="n">
         <v>2</v>
       </c>
     </row>
@@ -2220,18 +2374,23 @@
       </c>
       <c r="I20" t="inlineStr">
         <is>
+          <t>Principal C 9000000013</t>
+        </is>
+      </c>
+      <c r="J20" t="inlineStr">
+        <is>
           <t>Suresh 9000000008</t>
         </is>
       </c>
-      <c r="J20" t="n">
-        <v>2</v>
-      </c>
-      <c r="K20" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="M20" t="n">
+      <c r="K20" t="n">
+        <v>2</v>
+      </c>
+      <c r="L20" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="N20" t="n">
         <v>2</v>
       </c>
     </row>
@@ -2272,18 +2431,23 @@
       </c>
       <c r="I21" t="inlineStr">
         <is>
+          <t>Principal B 9000000012</t>
+        </is>
+      </c>
+      <c r="J21" t="inlineStr">
+        <is>
           <t>Lakshmi 9000000009</t>
         </is>
       </c>
-      <c r="J21" t="n">
-        <v>2</v>
-      </c>
-      <c r="K21" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="M21" t="n">
+      <c r="K21" t="n">
+        <v>2</v>
+      </c>
+      <c r="L21" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="N21" t="n">
         <v>2</v>
       </c>
     </row>
@@ -2324,18 +2488,23 @@
       </c>
       <c r="I22" t="inlineStr">
         <is>
+          <t>Principal C 9000000013</t>
+        </is>
+      </c>
+      <c r="J22" t="inlineStr">
+        <is>
           <t>Suresh 9000000008</t>
         </is>
       </c>
-      <c r="J22" t="n">
-        <v>2</v>
-      </c>
-      <c r="K22" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="M22" t="n">
+      <c r="K22" t="n">
+        <v>2</v>
+      </c>
+      <c r="L22" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="N22" t="n">
         <v>2</v>
       </c>
     </row>
@@ -2376,18 +2545,23 @@
       </c>
       <c r="I23" t="inlineStr">
         <is>
+          <t>Principal B 9000000012</t>
+        </is>
+      </c>
+      <c r="J23" t="inlineStr">
+        <is>
           <t>Lakshmi 9000000009</t>
         </is>
       </c>
-      <c r="J23" t="n">
-        <v>2</v>
-      </c>
-      <c r="K23" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="M23" t="n">
+      <c r="K23" t="n">
+        <v>2</v>
+      </c>
+      <c r="L23" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="N23" t="n">
         <v>2</v>
       </c>
     </row>
@@ -2428,18 +2602,23 @@
       </c>
       <c r="I24" t="inlineStr">
         <is>
+          <t>Principal C 9000000013</t>
+        </is>
+      </c>
+      <c r="J24" t="inlineStr">
+        <is>
           <t>Suresh 9000000008</t>
         </is>
       </c>
-      <c r="J24" t="n">
-        <v>2</v>
-      </c>
-      <c r="K24" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="M24" t="n">
+      <c r="K24" t="n">
+        <v>2</v>
+      </c>
+      <c r="L24" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="N24" t="n">
         <v>2</v>
       </c>
     </row>
@@ -2480,18 +2659,23 @@
       </c>
       <c r="I25" t="inlineStr">
         <is>
+          <t>Principal B 9000000012</t>
+        </is>
+      </c>
+      <c r="J25" t="inlineStr">
+        <is>
           <t>Lakshmi 9000000009</t>
         </is>
       </c>
-      <c r="J25" t="n">
-        <v>2</v>
-      </c>
-      <c r="K25" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="M25" t="n">
+      <c r="K25" t="n">
+        <v>2</v>
+      </c>
+      <c r="L25" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="N25" t="n">
         <v>2</v>
       </c>
     </row>
@@ -2532,18 +2716,23 @@
       </c>
       <c r="I26" t="inlineStr">
         <is>
+          <t>Principal C 9000000013</t>
+        </is>
+      </c>
+      <c r="J26" t="inlineStr">
+        <is>
           <t>Suresh 9000000008</t>
         </is>
       </c>
-      <c r="J26" t="n">
-        <v>2</v>
-      </c>
-      <c r="K26" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="M26" t="n">
+      <c r="K26" t="n">
+        <v>2</v>
+      </c>
+      <c r="L26" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="N26" t="n">
         <v>2</v>
       </c>
     </row>
@@ -2584,18 +2773,23 @@
       </c>
       <c r="I27" t="inlineStr">
         <is>
+          <t>Principal B 9000000012</t>
+        </is>
+      </c>
+      <c r="J27" t="inlineStr">
+        <is>
           <t>Lakshmi 9000000009</t>
         </is>
       </c>
-      <c r="J27" t="n">
-        <v>2</v>
-      </c>
-      <c r="K27" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="M27" t="n">
+      <c r="K27" t="n">
+        <v>2</v>
+      </c>
+      <c r="L27" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="N27" t="n">
         <v>2</v>
       </c>
     </row>
@@ -2636,18 +2830,23 @@
       </c>
       <c r="I28" t="inlineStr">
         <is>
+          <t>Principal C 9000000013</t>
+        </is>
+      </c>
+      <c r="J28" t="inlineStr">
+        <is>
           <t>Suresh 9000000008</t>
         </is>
       </c>
-      <c r="J28" t="n">
-        <v>2</v>
-      </c>
-      <c r="K28" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="M28" t="n">
+      <c r="K28" t="n">
+        <v>2</v>
+      </c>
+      <c r="L28" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="N28" t="n">
         <v>2</v>
       </c>
     </row>
@@ -2688,18 +2887,23 @@
       </c>
       <c r="I29" t="inlineStr">
         <is>
+          <t>Principal B 9000000012</t>
+        </is>
+      </c>
+      <c r="J29" t="inlineStr">
+        <is>
           <t>Lakshmi 9000000009</t>
         </is>
       </c>
-      <c r="J29" t="n">
-        <v>2</v>
-      </c>
-      <c r="K29" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="M29" t="n">
+      <c r="K29" t="n">
+        <v>2</v>
+      </c>
+      <c r="L29" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="N29" t="n">
         <v>2</v>
       </c>
     </row>
@@ -2740,24 +2944,29 @@
       </c>
       <c r="I30" t="inlineStr">
         <is>
+          <t>Principal A 9000000011</t>
+        </is>
+      </c>
+      <c r="J30" t="inlineStr">
+        <is>
           <t>Lakshmi 9000000009</t>
         </is>
       </c>
-      <c r="J30" t="n">
+      <c r="K30" t="n">
         <v>4</v>
       </c>
-      <c r="K30" t="inlineStr">
+      <c r="L30" t="inlineStr">
         <is>
           <t>Cancelled</t>
         </is>
       </c>
-      <c r="L30" s="7" t="inlineStr">
+      <c r="M30" s="7" t="inlineStr">
         <is>
           <t>Asha Rao 9000000001
 Ravi Kumar 9000000002 (via Asha Rao)</t>
         </is>
       </c>
-      <c r="M30" t="n">
+      <c r="N30" t="n">
         <v>2</v>
       </c>
     </row>
@@ -2798,18 +3007,23 @@
       </c>
       <c r="I31" t="inlineStr">
         <is>
+          <t>Principal B 9000000012</t>
+        </is>
+      </c>
+      <c r="J31" t="inlineStr">
+        <is>
           <t>Lakshmi 9000000009</t>
         </is>
       </c>
-      <c r="J31" t="n">
-        <v>2</v>
-      </c>
-      <c r="K31" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="M31" t="n">
+      <c r="K31" t="n">
+        <v>2</v>
+      </c>
+      <c r="L31" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="N31" t="n">
         <v>2</v>
       </c>
     </row>
@@ -2850,18 +3064,23 @@
       </c>
       <c r="I32" t="inlineStr">
         <is>
+          <t>Principal C 9000000013</t>
+        </is>
+      </c>
+      <c r="J32" t="inlineStr">
+        <is>
           <t>Suresh 9000000008</t>
         </is>
       </c>
-      <c r="J32" t="n">
-        <v>2</v>
-      </c>
-      <c r="K32" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="M32" t="n">
+      <c r="K32" t="n">
+        <v>2</v>
+      </c>
+      <c r="L32" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="N32" t="n">
         <v>2</v>
       </c>
     </row>
@@ -2902,18 +3121,23 @@
       </c>
       <c r="I33" t="inlineStr">
         <is>
+          <t>Principal C 9000000013</t>
+        </is>
+      </c>
+      <c r="J33" t="inlineStr">
+        <is>
           <t>Suresh 9000000008</t>
         </is>
       </c>
-      <c r="J33" t="n">
-        <v>2</v>
-      </c>
-      <c r="K33" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="M33" t="n">
+      <c r="K33" t="n">
+        <v>2</v>
+      </c>
+      <c r="L33" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="N33" t="n">
         <v>2</v>
       </c>
     </row>
@@ -2954,18 +3178,23 @@
       </c>
       <c r="I34" t="inlineStr">
         <is>
+          <t>Principal C 9000000013</t>
+        </is>
+      </c>
+      <c r="J34" t="inlineStr">
+        <is>
           <t>Suresh 9000000008</t>
         </is>
       </c>
-      <c r="J34" t="n">
-        <v>2</v>
-      </c>
-      <c r="K34" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="M34" t="n">
+      <c r="K34" t="n">
+        <v>2</v>
+      </c>
+      <c r="L34" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="N34" t="n">
         <v>2</v>
       </c>
     </row>
@@ -3006,18 +3235,23 @@
       </c>
       <c r="I35" t="inlineStr">
         <is>
+          <t>Principal C 9000000013</t>
+        </is>
+      </c>
+      <c r="J35" t="inlineStr">
+        <is>
           <t>Suresh 9000000008</t>
         </is>
       </c>
-      <c r="J35" t="n">
-        <v>2</v>
-      </c>
-      <c r="K35" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="M35" t="n">
+      <c r="K35" t="n">
+        <v>2</v>
+      </c>
+      <c r="L35" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="N35" t="n">
         <v>2</v>
       </c>
     </row>
@@ -3058,18 +3292,23 @@
       </c>
       <c r="I36" t="inlineStr">
         <is>
+          <t>Principal C 9000000013</t>
+        </is>
+      </c>
+      <c r="J36" t="inlineStr">
+        <is>
           <t>Suresh 9000000008</t>
         </is>
       </c>
-      <c r="J36" t="n">
-        <v>2</v>
-      </c>
-      <c r="K36" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="M36" t="n">
+      <c r="K36" t="n">
+        <v>2</v>
+      </c>
+      <c r="L36" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="N36" t="n">
         <v>2</v>
       </c>
     </row>
@@ -3110,24 +3349,29 @@
       </c>
       <c r="I37" t="inlineStr">
         <is>
+          <t>Principal A 9000000011</t>
+        </is>
+      </c>
+      <c r="J37" t="inlineStr">
+        <is>
           <t>Lakshmi 9000000009</t>
         </is>
       </c>
-      <c r="J37" t="n">
+      <c r="K37" t="n">
         <v>4</v>
       </c>
-      <c r="K37" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="L37" s="7" t="inlineStr">
+      <c r="L37" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="M37" s="7" t="inlineStr">
         <is>
           <t>Asha Rao 9000000001
 Ravi Kumar 9000000002 (via Asha Rao)</t>
         </is>
       </c>
-      <c r="M37" t="n">
+      <c r="N37" t="n">
         <v>2</v>
       </c>
     </row>
@@ -3168,18 +3412,23 @@
       </c>
       <c r="I38" t="inlineStr">
         <is>
+          <t>Principal D 9000000014</t>
+        </is>
+      </c>
+      <c r="J38" t="inlineStr">
+        <is>
           <t>Suresh 9000000008</t>
         </is>
       </c>
-      <c r="J38" t="n">
+      <c r="K38" t="n">
         <v>3</v>
       </c>
-      <c r="K38" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="M38" t="n">
+      <c r="L38" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="N38" t="n">
         <v>3</v>
       </c>
     </row>
@@ -3220,18 +3469,23 @@
       </c>
       <c r="I39" t="inlineStr">
         <is>
+          <t>Principal C 9000000013</t>
+        </is>
+      </c>
+      <c r="J39" t="inlineStr">
+        <is>
           <t>Suresh 9000000008</t>
         </is>
       </c>
-      <c r="J39" t="n">
-        <v>2</v>
-      </c>
-      <c r="K39" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="M39" t="n">
+      <c r="K39" t="n">
+        <v>2</v>
+      </c>
+      <c r="L39" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="N39" t="n">
         <v>2</v>
       </c>
     </row>
@@ -3272,18 +3526,23 @@
       </c>
       <c r="I40" t="inlineStr">
         <is>
+          <t>Principal C 9000000013</t>
+        </is>
+      </c>
+      <c r="J40" t="inlineStr">
+        <is>
           <t>Suresh 9000000008</t>
         </is>
       </c>
-      <c r="J40" t="n">
-        <v>2</v>
-      </c>
-      <c r="K40" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="M40" t="n">
+      <c r="K40" t="n">
+        <v>2</v>
+      </c>
+      <c r="L40" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="N40" t="n">
         <v>2</v>
       </c>
     </row>
@@ -3324,18 +3583,23 @@
       </c>
       <c r="I41" t="inlineStr">
         <is>
+          <t>Principal C 9000000013</t>
+        </is>
+      </c>
+      <c r="J41" t="inlineStr">
+        <is>
           <t>Suresh 9000000008</t>
         </is>
       </c>
-      <c r="J41" t="n">
-        <v>2</v>
-      </c>
-      <c r="K41" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="M41" t="n">
+      <c r="K41" t="n">
+        <v>2</v>
+      </c>
+      <c r="L41" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="N41" t="n">
         <v>2</v>
       </c>
     </row>
@@ -3376,18 +3640,23 @@
       </c>
       <c r="I42" t="inlineStr">
         <is>
+          <t>Principal C 9000000013</t>
+        </is>
+      </c>
+      <c r="J42" t="inlineStr">
+        <is>
           <t>Suresh 9000000008</t>
         </is>
       </c>
-      <c r="J42" t="n">
-        <v>2</v>
-      </c>
-      <c r="K42" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="M42" t="n">
+      <c r="K42" t="n">
+        <v>2</v>
+      </c>
+      <c r="L42" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="N42" t="n">
         <v>2</v>
       </c>
     </row>
@@ -3428,18 +3697,23 @@
       </c>
       <c r="I43" t="inlineStr">
         <is>
+          <t>Principal C 9000000013</t>
+        </is>
+      </c>
+      <c r="J43" t="inlineStr">
+        <is>
           <t>Suresh 9000000008</t>
         </is>
       </c>
-      <c r="J43" t="n">
-        <v>2</v>
-      </c>
-      <c r="K43" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="M43" t="n">
+      <c r="K43" t="n">
+        <v>2</v>
+      </c>
+      <c r="L43" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="N43" t="n">
         <v>2</v>
       </c>
     </row>
@@ -3480,18 +3754,23 @@
       </c>
       <c r="I44" t="inlineStr">
         <is>
+          <t>Principal A 9000000011</t>
+        </is>
+      </c>
+      <c r="J44" t="inlineStr">
+        <is>
           <t>Lakshmi 9000000009</t>
         </is>
       </c>
-      <c r="J44" t="n">
+      <c r="K44" t="n">
         <v>4</v>
       </c>
-      <c r="K44" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="M44" t="n">
+      <c r="L44" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="N44" t="n">
         <v>4</v>
       </c>
     </row>
@@ -3532,18 +3811,23 @@
       </c>
       <c r="I45" t="inlineStr">
         <is>
+          <t>Principal C 9000000013</t>
+        </is>
+      </c>
+      <c r="J45" t="inlineStr">
+        <is>
           <t>Suresh 9000000008</t>
         </is>
       </c>
-      <c r="J45" t="n">
-        <v>2</v>
-      </c>
-      <c r="K45" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="M45" t="n">
+      <c r="K45" t="n">
+        <v>2</v>
+      </c>
+      <c r="L45" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="N45" t="n">
         <v>2</v>
       </c>
     </row>
@@ -3584,18 +3868,23 @@
       </c>
       <c r="I46" t="inlineStr">
         <is>
+          <t>Principal C 9000000013</t>
+        </is>
+      </c>
+      <c r="J46" t="inlineStr">
+        <is>
           <t>Suresh 9000000008</t>
         </is>
       </c>
-      <c r="J46" t="n">
-        <v>2</v>
-      </c>
-      <c r="K46" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="M46" t="n">
+      <c r="K46" t="n">
+        <v>2</v>
+      </c>
+      <c r="L46" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="N46" t="n">
         <v>2</v>
       </c>
     </row>
@@ -3636,18 +3925,23 @@
       </c>
       <c r="I47" t="inlineStr">
         <is>
+          <t>Principal C 9000000013</t>
+        </is>
+      </c>
+      <c r="J47" t="inlineStr">
+        <is>
           <t>Suresh 9000000008</t>
         </is>
       </c>
-      <c r="J47" t="n">
-        <v>2</v>
-      </c>
-      <c r="K47" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="M47" t="n">
+      <c r="K47" t="n">
+        <v>2</v>
+      </c>
+      <c r="L47" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="N47" t="n">
         <v>2</v>
       </c>
     </row>
@@ -3688,18 +3982,23 @@
       </c>
       <c r="I48" t="inlineStr">
         <is>
+          <t>Principal C 9000000013</t>
+        </is>
+      </c>
+      <c r="J48" t="inlineStr">
+        <is>
           <t>Suresh 9000000008</t>
         </is>
       </c>
-      <c r="J48" t="n">
-        <v>2</v>
-      </c>
-      <c r="K48" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="M48" t="n">
+      <c r="K48" t="n">
+        <v>2</v>
+      </c>
+      <c r="L48" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="N48" t="n">
         <v>2</v>
       </c>
     </row>
@@ -3740,18 +4039,23 @@
       </c>
       <c r="I49" t="inlineStr">
         <is>
+          <t>Principal C 9000000013</t>
+        </is>
+      </c>
+      <c r="J49" t="inlineStr">
+        <is>
           <t>Suresh 9000000008</t>
         </is>
       </c>
-      <c r="J49" t="n">
-        <v>2</v>
-      </c>
-      <c r="K49" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="M49" t="n">
+      <c r="K49" t="n">
+        <v>2</v>
+      </c>
+      <c r="L49" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="N49" t="n">
         <v>2</v>
       </c>
     </row>
@@ -3787,18 +4091,23 @@
       </c>
       <c r="I50" t="inlineStr">
         <is>
+          <t>Principal G 9000000017</t>
+        </is>
+      </c>
+      <c r="J50" t="inlineStr">
+        <is>
           <t>Lakshmi 9000000009</t>
         </is>
       </c>
-      <c r="J50" t="n">
+      <c r="K50" t="n">
         <v>6</v>
       </c>
-      <c r="K50" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="M50" t="n">
+      <c r="L50" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="N50" t="n">
         <v>6</v>
       </c>
     </row>
@@ -3834,18 +4143,23 @@
       </c>
       <c r="I51" t="inlineStr">
         <is>
+          <t>Principal E 9000000015</t>
+        </is>
+      </c>
+      <c r="J51" t="inlineStr">
+        <is>
           <t>Lakshmi 9000000009</t>
         </is>
       </c>
-      <c r="J51" t="n">
+      <c r="K51" t="n">
         <v>5</v>
       </c>
-      <c r="K51" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="M51" t="n">
+      <c r="L51" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="N51" t="n">
         <v>5</v>
       </c>
     </row>
@@ -3886,18 +4200,23 @@
       </c>
       <c r="I52" t="inlineStr">
         <is>
+          <t>Principal A 9000000011</t>
+        </is>
+      </c>
+      <c r="J52" t="inlineStr">
+        <is>
           <t>Lakshmi 9000000009</t>
         </is>
       </c>
-      <c r="J52" t="n">
+      <c r="K52" t="n">
         <v>4</v>
       </c>
-      <c r="K52" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="M52" t="n">
+      <c r="L52" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="N52" t="n">
         <v>4</v>
       </c>
     </row>
@@ -3938,18 +4257,23 @@
       </c>
       <c r="I53" t="inlineStr">
         <is>
+          <t>Principal D 9000000014</t>
+        </is>
+      </c>
+      <c r="J53" t="inlineStr">
+        <is>
           <t>Suresh 9000000008</t>
         </is>
       </c>
-      <c r="J53" t="n">
+      <c r="K53" t="n">
         <v>3</v>
       </c>
-      <c r="K53" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="M53" t="n">
+      <c r="L53" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="N53" t="n">
         <v>3</v>
       </c>
     </row>
@@ -3985,18 +4309,23 @@
       </c>
       <c r="I54" t="inlineStr">
         <is>
+          <t>Principal F 9000000016</t>
+        </is>
+      </c>
+      <c r="J54" t="inlineStr">
+        <is>
           <t>Suresh 9000000008</t>
         </is>
       </c>
-      <c r="J54" t="n">
-        <v>2</v>
-      </c>
-      <c r="K54" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="M54" t="n">
+      <c r="K54" t="n">
+        <v>2</v>
+      </c>
+      <c r="L54" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="N54" t="n">
         <v>2</v>
       </c>
     </row>
@@ -4037,18 +4366,23 @@
       </c>
       <c r="I55" t="inlineStr">
         <is>
+          <t>Principal C 9000000013</t>
+        </is>
+      </c>
+      <c r="J55" t="inlineStr">
+        <is>
           <t>Suresh 9000000008</t>
         </is>
       </c>
-      <c r="J55" t="n">
-        <v>2</v>
-      </c>
-      <c r="K55" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="M55" t="n">
+      <c r="K55" t="n">
+        <v>2</v>
+      </c>
+      <c r="L55" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="N55" t="n">
         <v>2</v>
       </c>
     </row>
@@ -4089,18 +4423,23 @@
       </c>
       <c r="I56" t="inlineStr">
         <is>
+          <t>Principal C 9000000013</t>
+        </is>
+      </c>
+      <c r="J56" t="inlineStr">
+        <is>
           <t>Suresh 9000000008</t>
         </is>
       </c>
-      <c r="J56" t="n">
-        <v>2</v>
-      </c>
-      <c r="K56" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="M56" t="n">
+      <c r="K56" t="n">
+        <v>2</v>
+      </c>
+      <c r="L56" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="N56" t="n">
         <v>2</v>
       </c>
     </row>
@@ -4141,18 +4480,23 @@
       </c>
       <c r="I57" t="inlineStr">
         <is>
+          <t>Principal C 9000000013</t>
+        </is>
+      </c>
+      <c r="J57" t="inlineStr">
+        <is>
           <t>Suresh 9000000008</t>
         </is>
       </c>
-      <c r="J57" t="n">
-        <v>2</v>
-      </c>
-      <c r="K57" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="M57" t="n">
+      <c r="K57" t="n">
+        <v>2</v>
+      </c>
+      <c r="L57" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="N57" t="n">
         <v>2</v>
       </c>
     </row>
@@ -4193,18 +4537,23 @@
       </c>
       <c r="I58" t="inlineStr">
         <is>
+          <t>Principal C 9000000013</t>
+        </is>
+      </c>
+      <c r="J58" t="inlineStr">
+        <is>
           <t>Suresh 9000000008</t>
         </is>
       </c>
-      <c r="J58" t="n">
-        <v>2</v>
-      </c>
-      <c r="K58" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="M58" t="n">
+      <c r="K58" t="n">
+        <v>2</v>
+      </c>
+      <c r="L58" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="N58" t="n">
         <v>2</v>
       </c>
     </row>
@@ -4245,18 +4594,23 @@
       </c>
       <c r="I59" t="inlineStr">
         <is>
+          <t>Principal C 9000000013</t>
+        </is>
+      </c>
+      <c r="J59" t="inlineStr">
+        <is>
           <t>Suresh 9000000008</t>
         </is>
       </c>
-      <c r="J59" t="n">
-        <v>2</v>
-      </c>
-      <c r="K59" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="M59" t="n">
+      <c r="K59" t="n">
+        <v>2</v>
+      </c>
+      <c r="L59" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="N59" t="n">
         <v>2</v>
       </c>
     </row>
@@ -4297,18 +4651,23 @@
       </c>
       <c r="I60" t="inlineStr">
         <is>
+          <t>Principal A 9000000011</t>
+        </is>
+      </c>
+      <c r="J60" t="inlineStr">
+        <is>
           <t>Lakshmi 9000000009</t>
         </is>
       </c>
-      <c r="J60" t="n">
+      <c r="K60" t="n">
         <v>4</v>
       </c>
-      <c r="K60" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="M60" t="n">
+      <c r="L60" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="N60" t="n">
         <v>4</v>
       </c>
     </row>
@@ -4349,18 +4708,23 @@
       </c>
       <c r="I61" t="inlineStr">
         <is>
+          <t>Principal C 9000000013</t>
+        </is>
+      </c>
+      <c r="J61" t="inlineStr">
+        <is>
           <t>Suresh 9000000008</t>
         </is>
       </c>
-      <c r="J61" t="n">
-        <v>2</v>
-      </c>
-      <c r="K61" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="M61" t="n">
+      <c r="K61" t="n">
+        <v>2</v>
+      </c>
+      <c r="L61" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="N61" t="n">
         <v>2</v>
       </c>
     </row>
@@ -4401,18 +4765,23 @@
       </c>
       <c r="I62" t="inlineStr">
         <is>
+          <t>Principal C 9000000013</t>
+        </is>
+      </c>
+      <c r="J62" t="inlineStr">
+        <is>
           <t>Suresh 9000000008</t>
         </is>
       </c>
-      <c r="J62" t="n">
-        <v>2</v>
-      </c>
-      <c r="K62" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="M62" t="n">
+      <c r="K62" t="n">
+        <v>2</v>
+      </c>
+      <c r="L62" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="N62" t="n">
         <v>2</v>
       </c>
     </row>
@@ -4453,18 +4822,23 @@
       </c>
       <c r="I63" t="inlineStr">
         <is>
+          <t>Principal C 9000000013</t>
+        </is>
+      </c>
+      <c r="J63" t="inlineStr">
+        <is>
           <t>Suresh 9000000008</t>
         </is>
       </c>
-      <c r="J63" t="n">
-        <v>2</v>
-      </c>
-      <c r="K63" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="M63" t="n">
+      <c r="K63" t="n">
+        <v>2</v>
+      </c>
+      <c r="L63" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="N63" t="n">
         <v>2</v>
       </c>
     </row>
@@ -4505,18 +4879,23 @@
       </c>
       <c r="I64" t="inlineStr">
         <is>
+          <t>Principal C 9000000013</t>
+        </is>
+      </c>
+      <c r="J64" t="inlineStr">
+        <is>
           <t>Suresh 9000000008</t>
         </is>
       </c>
-      <c r="J64" t="n">
-        <v>2</v>
-      </c>
-      <c r="K64" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="M64" t="n">
+      <c r="K64" t="n">
+        <v>2</v>
+      </c>
+      <c r="L64" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="N64" t="n">
         <v>2</v>
       </c>
     </row>
@@ -4557,18 +4936,23 @@
       </c>
       <c r="I65" t="inlineStr">
         <is>
+          <t>Principal C 9000000013</t>
+        </is>
+      </c>
+      <c r="J65" t="inlineStr">
+        <is>
           <t>Suresh 9000000008</t>
         </is>
       </c>
-      <c r="J65" t="n">
-        <v>2</v>
-      </c>
-      <c r="K65" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="M65" t="n">
+      <c r="K65" t="n">
+        <v>2</v>
+      </c>
+      <c r="L65" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="N65" t="n">
         <v>2</v>
       </c>
     </row>
@@ -4609,18 +4993,23 @@
       </c>
       <c r="I66" t="inlineStr">
         <is>
+          <t>Principal A 9000000011</t>
+        </is>
+      </c>
+      <c r="J66" t="inlineStr">
+        <is>
           <t>Lakshmi 9000000009</t>
         </is>
       </c>
-      <c r="J66" t="n">
+      <c r="K66" t="n">
         <v>4</v>
       </c>
-      <c r="K66" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="M66" t="n">
+      <c r="L66" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="N66" t="n">
         <v>4</v>
       </c>
     </row>
@@ -4661,18 +5050,23 @@
       </c>
       <c r="I67" t="inlineStr">
         <is>
+          <t>Principal D 9000000014</t>
+        </is>
+      </c>
+      <c r="J67" t="inlineStr">
+        <is>
           <t>Suresh 9000000008</t>
         </is>
       </c>
-      <c r="J67" t="n">
+      <c r="K67" t="n">
         <v>3</v>
       </c>
-      <c r="K67" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="M67" t="n">
+      <c r="L67" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="N67" t="n">
         <v>3</v>
       </c>
     </row>
@@ -4713,18 +5107,23 @@
       </c>
       <c r="I68" t="inlineStr">
         <is>
+          <t>Principal C 9000000013</t>
+        </is>
+      </c>
+      <c r="J68" t="inlineStr">
+        <is>
           <t>Suresh 9000000008</t>
         </is>
       </c>
-      <c r="J68" t="n">
-        <v>2</v>
-      </c>
-      <c r="K68" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="M68" t="n">
+      <c r="K68" t="n">
+        <v>2</v>
+      </c>
+      <c r="L68" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="N68" t="n">
         <v>2</v>
       </c>
     </row>
@@ -4765,18 +5164,23 @@
       </c>
       <c r="I69" t="inlineStr">
         <is>
+          <t>Principal A 9000000011</t>
+        </is>
+      </c>
+      <c r="J69" t="inlineStr">
+        <is>
           <t>Lakshmi 9000000009</t>
         </is>
       </c>
-      <c r="J69" t="n">
+      <c r="K69" t="n">
         <v>4</v>
       </c>
-      <c r="K69" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="M69" t="n">
+      <c r="L69" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="N69" t="n">
         <v>4</v>
       </c>
     </row>
@@ -4812,18 +5216,23 @@
       </c>
       <c r="I70" t="inlineStr">
         <is>
+          <t>Principal E 9000000015</t>
+        </is>
+      </c>
+      <c r="J70" t="inlineStr">
+        <is>
           <t>Lakshmi 9000000009</t>
         </is>
       </c>
-      <c r="J70" t="n">
+      <c r="K70" t="n">
         <v>5</v>
       </c>
-      <c r="K70" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="M70" t="n">
+      <c r="L70" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="N70" t="n">
         <v>5</v>
       </c>
     </row>
@@ -4864,18 +5273,23 @@
       </c>
       <c r="I71" t="inlineStr">
         <is>
+          <t>Principal A 9000000011</t>
+        </is>
+      </c>
+      <c r="J71" t="inlineStr">
+        <is>
           <t>Lakshmi 9000000009</t>
         </is>
       </c>
-      <c r="J71" t="n">
+      <c r="K71" t="n">
         <v>4</v>
       </c>
-      <c r="K71" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="M71" t="n">
+      <c r="L71" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="N71" t="n">
         <v>4</v>
       </c>
     </row>
@@ -4916,18 +5330,23 @@
       </c>
       <c r="I72" t="inlineStr">
         <is>
+          <t>Principal D 9000000014</t>
+        </is>
+      </c>
+      <c r="J72" t="inlineStr">
+        <is>
           <t>Suresh 9000000008</t>
         </is>
       </c>
-      <c r="J72" t="n">
+      <c r="K72" t="n">
         <v>3</v>
       </c>
-      <c r="K72" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="M72" t="n">
+      <c r="L72" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="N72" t="n">
         <v>3</v>
       </c>
     </row>
@@ -4963,18 +5382,23 @@
       </c>
       <c r="I73" t="inlineStr">
         <is>
+          <t>Principal F 9000000016</t>
+        </is>
+      </c>
+      <c r="J73" t="inlineStr">
+        <is>
           <t>Suresh 9000000008</t>
         </is>
       </c>
-      <c r="J73" t="n">
-        <v>2</v>
-      </c>
-      <c r="K73" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="M73" t="n">
+      <c r="K73" t="n">
+        <v>2</v>
+      </c>
+      <c r="L73" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="N73" t="n">
         <v>2</v>
       </c>
     </row>
@@ -5015,18 +5439,23 @@
       </c>
       <c r="I74" t="inlineStr">
         <is>
+          <t>Principal A 9000000011</t>
+        </is>
+      </c>
+      <c r="J74" t="inlineStr">
+        <is>
           <t>Lakshmi 9000000009</t>
         </is>
       </c>
-      <c r="J74" t="n">
+      <c r="K74" t="n">
         <v>4</v>
       </c>
-      <c r="K74" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="M74" t="n">
+      <c r="L74" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="N74" t="n">
         <v>4</v>
       </c>
     </row>
@@ -5067,18 +5496,23 @@
       </c>
       <c r="I75" t="inlineStr">
         <is>
+          <t>Principal A 9000000011</t>
+        </is>
+      </c>
+      <c r="J75" t="inlineStr">
+        <is>
           <t>Lakshmi 9000000009</t>
         </is>
       </c>
-      <c r="J75" t="n">
+      <c r="K75" t="n">
         <v>4</v>
       </c>
-      <c r="K75" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="M75" t="n">
+      <c r="L75" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="N75" t="n">
         <v>4</v>
       </c>
     </row>
@@ -5119,18 +5553,23 @@
       </c>
       <c r="I76" t="inlineStr">
         <is>
+          <t>Principal D 9000000014</t>
+        </is>
+      </c>
+      <c r="J76" t="inlineStr">
+        <is>
           <t>Suresh 9000000008</t>
         </is>
       </c>
-      <c r="J76" t="n">
+      <c r="K76" t="n">
         <v>3</v>
       </c>
-      <c r="K76" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="M76" t="n">
+      <c r="L76" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="N76" t="n">
         <v>3</v>
       </c>
     </row>
@@ -5166,18 +5605,23 @@
       </c>
       <c r="I77" t="inlineStr">
         <is>
+          <t>Principal E 9000000015</t>
+        </is>
+      </c>
+      <c r="J77" t="inlineStr">
+        <is>
           <t>Lakshmi 9000000009</t>
         </is>
       </c>
-      <c r="J77" t="n">
+      <c r="K77" t="n">
         <v>5</v>
       </c>
-      <c r="K77" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="M77" t="n">
+      <c r="L77" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="N77" t="n">
         <v>5</v>
       </c>
     </row>
@@ -5213,18 +5657,23 @@
       </c>
       <c r="I78" t="inlineStr">
         <is>
+          <t>Principal F 9000000016</t>
+        </is>
+      </c>
+      <c r="J78" t="inlineStr">
+        <is>
           <t>Suresh 9000000008</t>
         </is>
       </c>
-      <c r="J78" t="n">
-        <v>2</v>
-      </c>
-      <c r="K78" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="M78" t="n">
+      <c r="K78" t="n">
+        <v>2</v>
+      </c>
+      <c r="L78" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="N78" t="n">
         <v>2</v>
       </c>
     </row>
@@ -5260,18 +5709,23 @@
       </c>
       <c r="I79" t="inlineStr">
         <is>
+          <t>Principal E 9000000015</t>
+        </is>
+      </c>
+      <c r="J79" t="inlineStr">
+        <is>
           <t>Lakshmi 9000000009</t>
         </is>
       </c>
-      <c r="J79" t="n">
+      <c r="K79" t="n">
         <v>5</v>
       </c>
-      <c r="K79" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="M79" t="n">
+      <c r="L79" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="N79" t="n">
         <v>5</v>
       </c>
     </row>
@@ -5307,18 +5761,23 @@
       </c>
       <c r="I80" t="inlineStr">
         <is>
+          <t>Principal F 9000000016</t>
+        </is>
+      </c>
+      <c r="J80" t="inlineStr">
+        <is>
           <t>Suresh 9000000008</t>
         </is>
       </c>
-      <c r="J80" t="n">
-        <v>2</v>
-      </c>
-      <c r="K80" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="M80" t="n">
+      <c r="K80" t="n">
+        <v>2</v>
+      </c>
+      <c r="L80" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="N80" t="n">
         <v>2</v>
       </c>
     </row>
@@ -5354,18 +5813,23 @@
       </c>
       <c r="I81" t="inlineStr">
         <is>
+          <t>Principal E 9000000015</t>
+        </is>
+      </c>
+      <c r="J81" t="inlineStr">
+        <is>
           <t>Lakshmi 9000000009</t>
         </is>
       </c>
-      <c r="J81" t="n">
+      <c r="K81" t="n">
         <v>5</v>
       </c>
-      <c r="K81" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="M81" t="n">
+      <c r="L81" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="N81" t="n">
         <v>5</v>
       </c>
     </row>
@@ -5401,24 +5865,29 @@
       </c>
       <c r="I82" t="inlineStr">
         <is>
+          <t>Principal F 9000000016</t>
+        </is>
+      </c>
+      <c r="J82" t="inlineStr">
+        <is>
           <t>Suresh 9000000008</t>
         </is>
       </c>
-      <c r="J82" t="n">
-        <v>2</v>
-      </c>
-      <c r="K82" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="M82" t="n">
+      <c r="K82" t="n">
+        <v>2</v>
+      </c>
+      <c r="L82" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="N82" t="n">
         <v>2</v>
       </c>
     </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation sqref="K2:K1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="L2:L1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>=Lists!$D$1:$D$2</formula1>
     </dataValidation>
   </dataValidations>
@@ -5671,7 +6140,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>last</t>
+          <t>5th</t>
         </is>
       </c>
     </row>
@@ -5684,6 +6153,11 @@
       <c r="B6" t="inlineStr">
         <is>
           <t>Monthly, same date</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>last</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Follow-up: Drive links first for the three demo videos (user, 2026-10-08); Week of month numbers only, 1st-5th, 'last' refused (user's choice); version followup-2026-10-08.5
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GfyZEqTUWy44eCLhgpngu7
</commit_message>
<xml_diff>
--- a/docs/followup/sample-followup-sheet.xlsx
+++ b/docs/followup/sample-followup-sheet.xlsx
@@ -184,7 +184,7 @@
     </comment>
     <comment ref="F1" authorId="0" shapeId="0">
       <text>
-        <t>Monthly, same weekday only: one of 1st, 2nd, 3rd, 4th, 5th (months without one are skipped) or last.</t>
+        <t>Monthly, same weekday only: one of 1st, 2nd, 3rd, 4th or 5th (months without a 5th are skipped).</t>
       </text>
     </comment>
     <comment ref="G1" authorId="0" shapeId="0">
@@ -1186,7 +1186,7 @@
       <formula1>=Lists!$B$1:$B$7</formula1>
     </dataValidation>
     <dataValidation sqref="F2:F1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>=Lists!$C$1:$C$6</formula1>
+      <formula1>=Lists!$C$1:$C$5</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -6155,11 +6155,6 @@
           <t>Monthly, same date</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>last</t>
-        </is>
-      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">

</xml_diff>